<commit_message>
file name fix and skipping exisiting files
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>bin</t>
+          <t>aaf</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>ajo7qz</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>db</t>
+          <t>asxqnd</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>db-shm</t>
+          <t>backup</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>db-wal</t>
+          <t>bin</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>exi</t>
+          <t>bw3lxx</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>exo</t>
+          <t>caffemodel</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>cfe</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>cfs</t>
         </is>
       </c>
     </row>
@@ -838,7 +838,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>obb</t>
+          <t>chck</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>pcache2</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
@@ -862,35 +862,406 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>config</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
         <is>
-          <t>tgs</t>
+          <t>crc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>tgv</t>
+          <t>crypt15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>tmp</t>
+          <t>dat</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
+          <t>db</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>db-journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>db-shm</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>db-wal</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>del</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>diffpak</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>eifs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>exi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>exo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fdt</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fdx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>flist</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>fnm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>hjvxdq</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>idx</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>info] 01 - chandamama nuvve nuvve</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>jwt</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>kwgt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>ltz</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>mdr</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>mega</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>mnn</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>mtthdt</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>nvd</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>nvm</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>obb</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>os</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>pak</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>pcache2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>pem</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>prototxt</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>replay</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>sav</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>temp</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>tgs</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>tgv</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>tmp</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>ttf</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71" t="inlineStr">
+        <is>
           <t>uid</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>vnf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: ADB download return code
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -489,11 +489,6 @@
           <t>avif</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>htm</t>
-        </is>
-      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>avi</t>
@@ -531,11 +526,6 @@
           <t>bmp</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>html</t>
-        </is>
-      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>flv</t>
@@ -568,11 +558,6 @@
           <t>gif</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>json</t>
-        </is>
-      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>mkv</t>
@@ -580,7 +565,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>aaf</t>
+          <t>bin</t>
         </is>
       </c>
     </row>
@@ -605,11 +590,6 @@
           <t>heic</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>md</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>mov</t>
@@ -617,7 +597,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ajo7qz</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
@@ -642,11 +622,6 @@
           <t>heif</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>sh</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>mp4</t>
@@ -654,7 +629,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>asxqnd</t>
+          <t>db</t>
         </is>
       </c>
     </row>
@@ -679,11 +654,6 @@
           <t>jfif</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>xml</t>
-        </is>
-      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>mpeg</t>
@@ -691,7 +661,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>backup</t>
+          <t>db-shm</t>
         </is>
       </c>
     </row>
@@ -723,7 +693,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>bin</t>
+          <t>db-wal</t>
         </is>
       </c>
     </row>
@@ -755,7 +725,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>bw3lxx</t>
+          <t>exi</t>
         </is>
       </c>
     </row>
@@ -787,7 +757,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>caffemodel</t>
+          <t>exo</t>
         </is>
       </c>
     </row>
@@ -809,7 +779,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>cfe</t>
+          <t>log</t>
         </is>
       </c>
     </row>
@@ -826,7 +796,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>cfs</t>
+          <t>m</t>
         </is>
       </c>
     </row>
@@ -838,7 +808,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>chck</t>
+          <t>obb</t>
         </is>
       </c>
     </row>
@@ -850,7 +820,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>pcache2</t>
         </is>
       </c>
     </row>
@@ -862,406 +832,42 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>prop</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
         <is>
-          <t>crc</t>
+          <t>sh</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>crypt15</t>
+          <t>tgs</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>dat</t>
+          <t>tgv</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
-          <t>db</t>
+          <t>tmp</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="H20" t="inlineStr">
         <is>
-          <t>db-journal</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>db-shm</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>db-wal</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>del</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>diffpak</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>eifs</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>exi</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>exo</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>fast</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>fdt</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>fdx</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>flist</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>fnm</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>full</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>gen</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>hjvxdq</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>idx</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>info</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>info] 01 - chandamama nuvve nuvve</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>ini</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>jwt</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>key</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>kwgt</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>log</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>ltz</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>mdr</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>mega</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>mnn</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>mtthdt</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>nvd</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>nvm</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>obb</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>os</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>pak</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>pcache2</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>pem</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>pos</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>prop</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>prototxt</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>replay</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>sav</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>temp</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>tgs</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>tgv</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>tim</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>tip</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>tmp</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>ttf</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="H71" t="inlineStr">
-        <is>
           <t>uid</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>vnf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: code cleanup & minor fixes
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -409,7 +409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>bin</t>
+          <t>aaf</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>ajo7qz</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>db</t>
+          <t>asxqnd</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>db-shm</t>
+          <t>backup</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>db-wal</t>
+          <t>bin</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>exi</t>
+          <t>bw3lxx</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>exo</t>
+          <t>caffemodel</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>cfe</t>
         </is>
       </c>
     </row>
@@ -796,7 +796,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>cfs</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>obb</t>
+          <t>chck</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>pcache2</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
@@ -832,42 +832,441 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>config</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
         <is>
-          <t>sh</t>
+          <t>crc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>tgs</t>
+          <t>crypt15</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>tgv</t>
+          <t>dat</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
-          <t>tmp</t>
+          <t>db</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="H20" t="inlineStr">
         <is>
+          <t>db-journal</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>db-shm</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>db-wal</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>del</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>diffpak</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>eifs</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>exi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>exo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>fast</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>fdt</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fdx</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>flist</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>fnm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>gen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>hjvxdq</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>idx</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>info] 01 - chandamama nuvve nuvve</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>jwt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>kwgt</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>ltz</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>mdr</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>mega</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>mnn</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>mtthdt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>nvd</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>nvm</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>obb</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>os</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>pak</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>pcache2</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>pem</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>preload</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>prototxt</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>replay</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>sav</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>temp</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>tgs</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>tgv</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>tmp</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>ttf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="H75" t="inlineStr">
+        <is>
           <t>uid</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>vnf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>xml</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bug fix: ADB add path
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>jpf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>png</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -769,7 +769,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>tif</t>
+          <t>svg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>tiff</t>
+          <t>tif</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -798,16 +798,21 @@
     <row r="13">
       <c r="E13" t="inlineStr">
         <is>
+          <t>tiff</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>chck</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" t="inlineStr">
+        <is>
           <t>webp</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>chck</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
       <c r="H14" t="inlineStr">
         <is>
           <t>clean</t>

</xml_diff>

<commit_message>
ADB Environment Path fix
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -409,7 +409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="4.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -565,7 +565,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>aaf</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>ajo7qz</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>asxqnd</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>jpeg</t>
+          <t>jfif</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>backup</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>jpf</t>
+          <t>jpeg</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>bin</t>
+          <t>aaf</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>jpf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>bw3lxx</t>
+          <t>ajo7qz</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>caffemodel</t>
+          <t>aspx</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>png</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>cfe</t>
+          <t>asxqnd</t>
         </is>
       </c>
     </row>
@@ -786,482 +786,620 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>tif</t>
+          <t>svg</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>cfs</t>
+          <t>backup</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="E13" t="inlineStr">
         <is>
-          <t>tiff</t>
+          <t>tif</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>chck</t>
+          <t>bin</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="E14" t="inlineStr">
         <is>
+          <t>tiff</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="inlineStr">
+        <is>
           <t>webp</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>clean</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
       <c r="H15" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>bw3lxx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
         <is>
-          <t>crc</t>
+          <t>cache</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>crypt15</t>
+          <t>caffemodel</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>dat</t>
+          <t>cfe</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
-          <t>db</t>
+          <t>cfs</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="H20" t="inlineStr">
         <is>
-          <t>db-journal</t>
+          <t>chck</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="H21" t="inlineStr">
         <is>
-          <t>db-shm</t>
+          <t>checksum</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="H22" t="inlineStr">
         <is>
-          <t>db-wal</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="H23" t="inlineStr">
         <is>
-          <t>del</t>
+          <t>config</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="H24" t="inlineStr">
         <is>
-          <t>diffpak</t>
+          <t>crc</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="H25" t="inlineStr">
         <is>
-          <t>eifs</t>
+          <t>crypt15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="H26" t="inlineStr">
         <is>
-          <t>exi</t>
+          <t>css</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="H27" t="inlineStr">
         <is>
-          <t>exo</t>
+          <t>dat</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="H28" t="inlineStr">
         <is>
-          <t>fast</t>
+          <t>db</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="H29" t="inlineStr">
         <is>
-          <t>fdt</t>
+          <t>db-journal</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="H30" t="inlineStr">
         <is>
-          <t>fdx</t>
+          <t>db-shm</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="H31" t="inlineStr">
         <is>
-          <t>flist</t>
+          <t>db-wal</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="H32" t="inlineStr">
         <is>
-          <t>fnm</t>
+          <t>del</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="H33" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>diffpak</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="H34" t="inlineStr">
         <is>
-          <t>gen</t>
+          <t>eifs</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="H35" t="inlineStr">
         <is>
-          <t>hjvxdq</t>
+          <t>exi</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="H36" t="inlineStr">
         <is>
-          <t>idx</t>
+          <t>exo</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="H37" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>fast</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="H38" t="inlineStr">
         <is>
-          <t>info] 01 - chandamama nuvve nuvve</t>
+          <t>fdt</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="H39" t="inlineStr">
         <is>
-          <t>ini</t>
+          <t>fdx</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="H40" t="inlineStr">
         <is>
-          <t>jfif</t>
+          <t>flist</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="H41" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>fnm</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="H42" t="inlineStr">
         <is>
-          <t>jwt</t>
+          <t>full</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="H43" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>gen</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="H44" t="inlineStr">
         <is>
-          <t>kwgt</t>
+          <t>hjvxdq</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="H45" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>html</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="H46" t="inlineStr">
         <is>
-          <t>ltz</t>
+          <t>idx</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="H47" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>info</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="H48" t="inlineStr">
         <is>
-          <t>mdr</t>
+          <t>info] 01 - chandamama nuvve nuvve</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="H49" t="inlineStr">
         <is>
-          <t>mega</t>
+          <t>ini</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="H50" t="inlineStr">
         <is>
-          <t>mnn</t>
+          <t>js</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="H51" t="inlineStr">
         <is>
-          <t>mtthdt</t>
+          <t>json</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="H52" t="inlineStr">
         <is>
-          <t>nvd</t>
+          <t>jwt</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="H53" t="inlineStr">
         <is>
-          <t>nvm</t>
+          <t>key</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="H54" t="inlineStr">
         <is>
-          <t>obb</t>
+          <t>kva</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="H55" t="inlineStr">
         <is>
-          <t>os</t>
+          <t>kvb</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="H56" t="inlineStr">
         <is>
-          <t>pak</t>
+          <t>kwgt</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="H57" t="inlineStr">
         <is>
-          <t>pcache2</t>
+          <t>log</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="H58" t="inlineStr">
         <is>
-          <t>pem</t>
+          <t>ltz</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="H59" t="inlineStr">
         <is>
-          <t>pos</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="H60" t="inlineStr">
         <is>
-          <t>preload</t>
+          <t>map</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="H61" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>mdr</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="H62" t="inlineStr">
         <is>
-          <t>prototxt</t>
+          <t>mega</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="H63" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>meta</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="H64" t="inlineStr">
         <is>
-          <t>replay</t>
+          <t>mmap</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="H65" t="inlineStr">
         <is>
-          <t>res</t>
+          <t>mnn</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="H66" t="inlineStr">
         <is>
-          <t>sav</t>
+          <t>mtthdt</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="H67" t="inlineStr">
         <is>
-          <t>sh</t>
+          <t>nvd</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="H68" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>nvm</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="H69" t="inlineStr">
         <is>
-          <t>temp</t>
+          <t>obb</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="H70" t="inlineStr">
         <is>
-          <t>tgs</t>
+          <t>os</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="H71" t="inlineStr">
         <is>
-          <t>tgv</t>
+          <t>pak</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="H72" t="inlineStr">
         <is>
-          <t>tim</t>
+          <t>pcache2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="H73" t="inlineStr">
         <is>
-          <t>tip</t>
+          <t>pdb</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="H74" t="inlineStr">
         <is>
-          <t>tmp</t>
+          <t>pem</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="H75" t="inlineStr">
         <is>
-          <t>ttf</t>
+          <t>pos</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="H76" t="inlineStr">
         <is>
-          <t>uid</t>
+          <t>preload</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="H77" t="inlineStr">
         <is>
-          <t>vnf</t>
+          <t>prop</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="H78" t="inlineStr">
+        <is>
+          <t>prototxt</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>pt</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>replay</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>sav</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>sna</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>temp</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>tgs</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>tgv</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>tmp</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>torrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>ttf</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>uid</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>vnf</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="H97" t="inlineStr">
         <is>
           <t>xml</t>
         </is>

</xml_diff>

<commit_message>
Removed env from Repo
</commit_message>
<xml_diff>
--- a/data/categories.xlsx
+++ b/data/categories.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -409,16 +409,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H108"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="4.88671875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="7.77734375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="5.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="10.21875" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6.77734375" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="6.44140625" bestFit="1" customWidth="1" min="6" max="7"/>
-    <col width="7.21875" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="4.90625" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="7.81640625" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="5.6328125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="10.1796875" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="6.81640625" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="6.453125" bestFit="1" customWidth="1" min="6" max="7"/>
+    <col width="7.1796875" bestFit="1" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="1">
@@ -565,7 +565,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>aaf</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>ajo7qz</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>asc</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>jfif</t>
+          <t>jpeg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>aspx</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>jpeg</t>
+          <t>jpf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>aaf</t>
+          <t>ast</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>jpf</t>
+          <t>jpg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>ajo7qz</t>
+          <t>asxqnd</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>jpg</t>
+          <t>png</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>aspx</t>
+          <t>backup</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>png</t>
+          <t>svg</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>asxqnd</t>
+          <t>bin</t>
         </is>
       </c>
     </row>
@@ -786,174 +786,169 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>svg</t>
+          <t>tif</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>backup</t>
+          <t>blog</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="E13" t="inlineStr">
         <is>
-          <t>tif</t>
+          <t>tiff</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>bin</t>
+          <t>browser</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="E14" t="inlineStr">
         <is>
-          <t>tiff</t>
+          <t>webp</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>browser</t>
+          <t>bw3lxx</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>webp</t>
-        </is>
-      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>bw3lxx</t>
+          <t>cache</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="H16" t="inlineStr">
         <is>
-          <t>cache</t>
+          <t>caffemodel</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="H17" t="inlineStr">
         <is>
-          <t>caffemodel</t>
+          <t>cfe</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="H18" t="inlineStr">
         <is>
-          <t>cfe</t>
+          <t>cfs</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="H19" t="inlineStr">
         <is>
-          <t>cfs</t>
+          <t>chck</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="H20" t="inlineStr">
         <is>
-          <t>chck</t>
+          <t>checksum</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="H21" t="inlineStr">
         <is>
-          <t>checksum</t>
+          <t>clean</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="H22" t="inlineStr">
         <is>
-          <t>clean</t>
+          <t>config</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="H23" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>crc</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="H24" t="inlineStr">
         <is>
-          <t>crc</t>
+          <t>crypt15</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="H25" t="inlineStr">
         <is>
-          <t>crypt15</t>
+          <t>css</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="H26" t="inlineStr">
         <is>
-          <t>css</t>
+          <t>dat</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="H27" t="inlineStr">
         <is>
-          <t>dat</t>
+          <t>db</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="H28" t="inlineStr">
         <is>
-          <t>db</t>
+          <t>db-journal</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="H29" t="inlineStr">
         <is>
-          <t>db-journal</t>
+          <t>db-shm</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="H30" t="inlineStr">
         <is>
-          <t>db-shm</t>
+          <t>db-wal</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="H31" t="inlineStr">
         <is>
-          <t>db-wal</t>
+          <t>del</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="H32" t="inlineStr">
         <is>
-          <t>del</t>
+          <t>diffpak</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="H33" t="inlineStr">
         <is>
-          <t>diffpak</t>
+          <t>ds_store</t>
         </is>
       </c>
     </row>
@@ -1051,355 +1046,432 @@
     <row r="47">
       <c r="H47" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>img</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="H48" t="inlineStr">
         <is>
-          <t>info] 01 - chandamama nuvve nuvve</t>
+          <t>info</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="H49" t="inlineStr">
         <is>
-          <t>ini</t>
+          <t>info] 01 - chandamama nuvve nuvve</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="H50" t="inlineStr">
         <is>
-          <t>js</t>
+          <t>ini</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="H51" t="inlineStr">
         <is>
-          <t>json</t>
+          <t>jfif</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="H52" t="inlineStr">
         <is>
-          <t>jwt</t>
+          <t>js</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="H53" t="inlineStr">
         <is>
-          <t>key</t>
+          <t>json</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="H54" t="inlineStr">
         <is>
-          <t>kva</t>
+          <t>jwt</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="H55" t="inlineStr">
         <is>
-          <t>kvb</t>
+          <t>key</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="H56" t="inlineStr">
         <is>
-          <t>kwgt</t>
+          <t>kfx</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="H57" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>kva</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="H58" t="inlineStr">
         <is>
-          <t>ltz</t>
+          <t>kvb</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="H59" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kwgt</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="H60" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>log</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="H61" t="inlineStr">
         <is>
-          <t>mdr</t>
+          <t>ltz</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="H62" t="inlineStr">
         <is>
-          <t>mega</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="H63" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>map</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="H64" t="inlineStr">
         <is>
-          <t>mmap</t>
+          <t>mdr</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="H65" t="inlineStr">
         <is>
-          <t>mnn</t>
+          <t>mega</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="H66" t="inlineStr">
         <is>
-          <t>mtthdt</t>
+          <t>meta</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="H67" t="inlineStr">
         <is>
-          <t>nvd</t>
+          <t>min</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="H68" t="inlineStr">
         <is>
-          <t>nvm</t>
+          <t>mmap</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="H69" t="inlineStr">
         <is>
-          <t>obb</t>
+          <t>mnn</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="H70" t="inlineStr">
         <is>
-          <t>os</t>
+          <t>mtthdt</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="H71" t="inlineStr">
         <is>
-          <t>pak</t>
+          <t>nvd</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="H72" t="inlineStr">
         <is>
-          <t>pcache2</t>
+          <t>nvm</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="H73" t="inlineStr">
         <is>
-          <t>pdb</t>
+          <t>obb</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="H74" t="inlineStr">
         <is>
-          <t>pem</t>
+          <t>os</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="H75" t="inlineStr">
         <is>
-          <t>pos</t>
+          <t>otf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="H76" t="inlineStr">
         <is>
-          <t>preload</t>
+          <t>pak</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="H77" t="inlineStr">
         <is>
-          <t>prop</t>
+          <t>pcache2</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="H78" t="inlineStr">
         <is>
-          <t>prototxt</t>
+          <t>pdb</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="H79" t="inlineStr">
         <is>
-          <t>pt</t>
+          <t>pem</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="H80" t="inlineStr">
         <is>
-          <t>replay</t>
+          <t>phl</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="H81" t="inlineStr">
         <is>
-          <t>res</t>
+          <t>pos</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="H82" t="inlineStr">
         <is>
-          <t>sav</t>
+          <t>preload</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="H83" t="inlineStr">
         <is>
-          <t>sh</t>
+          <t>prop</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="H84" t="inlineStr">
         <is>
-          <t>si</t>
+          <t>prototxt</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="H85" t="inlineStr">
         <is>
-          <t>sna</t>
+          <t>pt</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="H86" t="inlineStr">
         <is>
-          <t>temp</t>
+          <t>py</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="H87" t="inlineStr">
         <is>
-          <t>tgs</t>
+          <t>replay</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="H88" t="inlineStr">
         <is>
-          <t>tgv</t>
+          <t>res</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="H89" t="inlineStr">
         <is>
-          <t>tim</t>
+          <t>sav</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="H90" t="inlineStr">
         <is>
-          <t>tip</t>
+          <t>ser</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="H91" t="inlineStr">
         <is>
-          <t>tmp</t>
+          <t>sh</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="H92" t="inlineStr">
         <is>
-          <t>torrent</t>
+          <t>si</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="H93" t="inlineStr">
         <is>
-          <t>ttf</t>
+          <t>sna</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="H94" t="inlineStr">
         <is>
-          <t>uid</t>
+          <t>srt</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="H95" t="inlineStr">
         <is>
-          <t>ver</t>
+          <t>temp</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="H96" t="inlineStr">
         <is>
-          <t>vnf</t>
+          <t>tgs</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="H97" t="inlineStr">
+        <is>
+          <t>tgv</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>ticr</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>tim</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>tmp</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>torrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>ttf</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>uid</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>vnf</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>vng_meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="H108" t="inlineStr">
         <is>
           <t>xml</t>
         </is>

</xml_diff>